<commit_message>
- Add hds-forms-model-lib to settings.gradle - Update forms ext_inmigration_form.xlsx, member_enu_form.xlsx, and inmigration_form.xlsx to put dummy education, religion options (theyre loaded externally)
</commit_message>
<xml_diff>
--- a/app/src/main/res/raw/ext_inmigration_form.xlsx
+++ b/app/src/main/res/raw/ext_inmigration_form.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27795" windowHeight="12195" tabRatio="500"/>
+    <workbookView windowWidth="24090" windowHeight="11400" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="columns" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="323">
   <si>
     <t>group</t>
   </si>
@@ -992,6 +992,9 @@
   </si>
   <si>
     <t xml:space="preserve">አላውቅም </t>
+  </si>
+  <si>
+    <t>LOADED_EXTERNALLY</t>
   </si>
   <si>
     <t>form_id</t>
@@ -1023,10 +1026,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="27">
     <font>
@@ -1060,15 +1063,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1083,23 +1080,44 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="18"/>
+      <sz val="15"/>
       <color theme="3"/>
       <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1113,54 +1131,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF006100"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1181,16 +1161,40 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
-      <sz val="15"/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
       <color theme="3"/>
       <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1203,11 +1207,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1243,7 +1246,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1261,7 +1270,109 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1273,19 +1384,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1303,25 +1408,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1333,97 +1426,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1501,6 +1504,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="double">
         <color rgb="FF3F3F3F"/>
       </left>
@@ -1516,6 +1528,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -1527,21 +1548,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1563,15 +1569,6 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
@@ -1581,11 +1578,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1601,152 +1604,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1772,13 +1775,18 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1790,7 +1798,7 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1801,7 +1809,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2214,7 +2221,7 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="30" t="s">
+      <c r="J1" s="32" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
@@ -2232,7 +2239,7 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="44" t="s">
+      <c r="P1" s="46" t="s">
         <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
@@ -2248,24 +2255,24 @@
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="15" t="s">
         <v>20</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="12" t="s">
+      <c r="H2" s="15" t="s">
         <v>21</v>
       </c>
       <c r="I2" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="31" t="s">
+      <c r="J2" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="12" t="s">
+      <c r="K2" s="15" t="s">
         <v>24</v>
       </c>
       <c r="L2" s="1"/>
@@ -2276,7 +2283,7 @@
       <c r="O2" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="P2" s="44"/>
+      <c r="P2" s="46"/>
     </row>
     <row r="3" spans="1:15">
       <c r="A3" s="1" t="s">
@@ -2294,14 +2301,14 @@
       <c r="I3" t="s">
         <v>27</v>
       </c>
-      <c r="J3" s="31" t="s">
+      <c r="J3" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="K3" s="32" t="s">
+      <c r="K3" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="L3" s="33"/>
-      <c r="M3" s="33"/>
+      <c r="L3" s="35"/>
+      <c r="M3" s="35"/>
       <c r="N3" t="b">
         <v>1</v>
       </c>
@@ -2325,14 +2332,14 @@
       <c r="I4" t="s">
         <v>33</v>
       </c>
-      <c r="J4" s="31" t="s">
+      <c r="J4" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="K4" s="32" t="s">
+      <c r="K4" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="L4" s="33"/>
-      <c r="M4" s="33"/>
+      <c r="L4" s="35"/>
+      <c r="M4" s="35"/>
       <c r="N4" t="b">
         <v>1</v>
       </c>
@@ -2358,14 +2365,14 @@
       <c r="I5" t="s">
         <v>38</v>
       </c>
-      <c r="J5" s="31" t="s">
+      <c r="J5" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="K5" s="32" t="s">
+      <c r="K5" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="L5" s="33"/>
-      <c r="M5" s="33"/>
+      <c r="L5" s="35"/>
+      <c r="M5" s="35"/>
       <c r="N5" t="b">
         <v>1</v>
       </c>
@@ -2389,14 +2396,14 @@
       <c r="I6" t="s">
         <v>43</v>
       </c>
-      <c r="J6" s="31" t="s">
+      <c r="J6" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="K6" s="32" t="s">
+      <c r="K6" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="L6" s="33"/>
-      <c r="M6" s="33"/>
+      <c r="L6" s="35"/>
+      <c r="M6" s="35"/>
       <c r="N6" t="b">
         <v>1</v>
       </c>
@@ -2420,14 +2427,14 @@
       <c r="I7" t="s">
         <v>48</v>
       </c>
-      <c r="J7" s="31" t="s">
+      <c r="J7" s="33" t="s">
         <v>49</v>
       </c>
-      <c r="K7" s="32" t="s">
+      <c r="K7" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="L7" s="33"/>
-      <c r="M7" s="33"/>
+      <c r="L7" s="35"/>
+      <c r="M7" s="35"/>
       <c r="N7" t="b">
         <v>1</v>
       </c>
@@ -2454,14 +2461,14 @@
       <c r="I8" t="s">
         <v>56</v>
       </c>
-      <c r="J8" s="31" t="s">
+      <c r="J8" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="K8" s="32" t="s">
+      <c r="K8" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="L8" s="33"/>
-      <c r="M8" s="33"/>
+      <c r="L8" s="35"/>
+      <c r="M8" s="35"/>
       <c r="N8" t="b">
         <v>1</v>
       </c>
@@ -2491,14 +2498,14 @@
       <c r="I9" t="s">
         <v>63</v>
       </c>
-      <c r="J9" s="31" t="s">
+      <c r="J9" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="K9" s="32" t="s">
+      <c r="K9" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="L9" s="33"/>
-      <c r="M9" s="33"/>
+      <c r="L9" s="35"/>
+      <c r="M9" s="35"/>
       <c r="N9" t="b">
         <v>1</v>
       </c>
@@ -2525,14 +2532,14 @@
       <c r="I10" t="s">
         <v>69</v>
       </c>
-      <c r="J10" s="31" t="s">
+      <c r="J10" s="33" t="s">
         <v>70</v>
       </c>
-      <c r="K10" s="32" t="s">
+      <c r="K10" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="L10" s="33"/>
-      <c r="M10" s="33"/>
+      <c r="L10" s="35"/>
+      <c r="M10" s="35"/>
       <c r="N10" t="b">
         <v>1</v>
       </c>
@@ -2556,14 +2563,14 @@
       <c r="I11" t="s">
         <v>76</v>
       </c>
-      <c r="J11" s="31" t="s">
+      <c r="J11" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="K11" s="32" t="s">
+      <c r="K11" s="34" t="s">
         <v>78</v>
       </c>
-      <c r="L11" s="33"/>
-      <c r="M11" s="33"/>
+      <c r="L11" s="35"/>
+      <c r="M11" s="35"/>
       <c r="N11" t="b">
         <v>1</v>
       </c>
@@ -2585,14 +2592,14 @@
       <c r="I12" t="s">
         <v>82</v>
       </c>
-      <c r="J12" s="31" t="s">
+      <c r="J12" s="33" t="s">
         <v>83</v>
       </c>
-      <c r="K12" s="32" t="s">
+      <c r="K12" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="L12" s="33"/>
-      <c r="M12" s="33"/>
+      <c r="L12" s="35"/>
+      <c r="M12" s="35"/>
       <c r="N12" t="b">
         <v>1</v>
       </c>
@@ -2617,18 +2624,18 @@
       <c r="I13" t="s">
         <v>88</v>
       </c>
-      <c r="J13" s="31" t="s">
+      <c r="J13" s="33" t="s">
         <v>89</v>
       </c>
-      <c r="K13" s="32" t="s">
+      <c r="K13" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="L13" s="33"/>
-      <c r="M13" s="33"/>
+      <c r="L13" s="35"/>
+      <c r="M13" s="35"/>
       <c r="N13" t="b">
         <v>1</v>
       </c>
-      <c r="P13" s="45" t="s">
+      <c r="P13" s="47" t="s">
         <v>91</v>
       </c>
     </row>
@@ -2646,14 +2653,14 @@
       <c r="I14" t="s">
         <v>94</v>
       </c>
-      <c r="J14" s="31" t="s">
+      <c r="J14" s="33" t="s">
         <v>95</v>
       </c>
-      <c r="K14" s="32" t="s">
+      <c r="K14" s="34" t="s">
         <v>96</v>
       </c>
-      <c r="L14" s="33"/>
-      <c r="M14" s="33"/>
+      <c r="L14" s="35"/>
+      <c r="M14" s="35"/>
       <c r="N14" t="b">
         <v>1</v>
       </c>
@@ -2678,14 +2685,14 @@
       <c r="I15" t="s">
         <v>99</v>
       </c>
-      <c r="J15" s="31" t="s">
+      <c r="J15" s="33" t="s">
         <v>100</v>
       </c>
-      <c r="K15" s="32" t="s">
+      <c r="K15" s="34" t="s">
         <v>101</v>
       </c>
-      <c r="L15" s="33"/>
-      <c r="M15" s="33"/>
+      <c r="L15" s="35"/>
+      <c r="M15" s="35"/>
       <c r="N15" t="b">
         <v>1</v>
       </c>
@@ -2707,14 +2714,14 @@
       <c r="I16" t="s">
         <v>104</v>
       </c>
-      <c r="J16" s="31" t="s">
+      <c r="J16" s="33" t="s">
         <v>105</v>
       </c>
-      <c r="K16" s="32" t="s">
+      <c r="K16" s="34" t="s">
         <v>106</v>
       </c>
-      <c r="L16" s="33"/>
-      <c r="M16" s="33"/>
+      <c r="L16" s="35"/>
+      <c r="M16" s="35"/>
       <c r="N16" t="b">
         <v>1</v>
       </c>
@@ -2736,14 +2743,14 @@
       <c r="I17" t="s">
         <v>109</v>
       </c>
-      <c r="J17" s="31" t="s">
+      <c r="J17" s="33" t="s">
         <v>110</v>
       </c>
-      <c r="K17" s="32" t="s">
+      <c r="K17" s="34" t="s">
         <v>111</v>
       </c>
-      <c r="L17" s="33"/>
-      <c r="M17" s="33"/>
+      <c r="L17" s="35"/>
+      <c r="M17" s="35"/>
       <c r="N17" t="b">
         <v>1</v>
       </c>
@@ -2765,14 +2772,14 @@
       <c r="I18" t="s">
         <v>115</v>
       </c>
-      <c r="J18" s="31" t="s">
+      <c r="J18" s="33" t="s">
         <v>116</v>
       </c>
-      <c r="K18" s="32" t="s">
+      <c r="K18" s="34" t="s">
         <v>117</v>
       </c>
-      <c r="L18" s="33"/>
-      <c r="M18" s="33"/>
+      <c r="L18" s="35"/>
+      <c r="M18" s="35"/>
       <c r="N18" t="b">
         <v>1</v>
       </c>
@@ -2791,14 +2798,14 @@
       <c r="I19" t="s">
         <v>120</v>
       </c>
-      <c r="J19" s="31" t="s">
+      <c r="J19" s="33" t="s">
         <v>121</v>
       </c>
-      <c r="K19" s="32" t="s">
+      <c r="K19" s="34" t="s">
         <v>122</v>
       </c>
-      <c r="L19" s="33"/>
-      <c r="M19" s="33"/>
+      <c r="L19" s="35"/>
+      <c r="M19" s="35"/>
       <c r="N19" t="b">
         <v>1</v>
       </c>
@@ -2807,380 +2814,380 @@
       </c>
     </row>
     <row r="20" spans="1:18">
-      <c r="A20" s="23"/>
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24" t="s">
+      <c r="A20" s="26"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="E20" s="24" t="s">
+      <c r="E20" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="F20" s="24" t="s">
+      <c r="F20" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24" t="s">
+      <c r="G20" s="11"/>
+      <c r="H20" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="I20" s="24" t="s">
+      <c r="I20" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="J20" s="24" t="s">
+      <c r="J20" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="K20" s="34" t="s">
+      <c r="K20" s="36" t="s">
         <v>129</v>
       </c>
-      <c r="L20" s="35"/>
-      <c r="M20" s="35"/>
-      <c r="N20" s="24" t="b">
-        <v>1</v>
-      </c>
-      <c r="O20" s="24"/>
-      <c r="P20" s="24" t="s">
+      <c r="L20" s="37"/>
+      <c r="M20" s="37"/>
+      <c r="N20" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="O20" s="11"/>
+      <c r="P20" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="Q20" s="24"/>
-      <c r="R20" s="24"/>
+      <c r="Q20" s="11"/>
+      <c r="R20" s="11"/>
     </row>
     <row r="21" spans="1:18">
-      <c r="A21" s="23"/>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24" t="s">
+      <c r="A21" s="26"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="E21" s="24" t="s">
+      <c r="E21" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="F21" s="24" t="s">
+      <c r="F21" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="G21" s="24"/>
-      <c r="H21" s="24" t="s">
+      <c r="G21" s="11"/>
+      <c r="H21" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="I21" s="24" t="s">
+      <c r="I21" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="J21" s="24" t="s">
+      <c r="J21" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="K21" s="34" t="s">
+      <c r="K21" s="36" t="s">
         <v>135</v>
       </c>
-      <c r="L21" s="35"/>
-      <c r="M21" s="35"/>
-      <c r="N21" s="24" t="b">
-        <v>1</v>
-      </c>
-      <c r="O21" s="24"/>
-      <c r="P21" s="24"/>
-      <c r="Q21" s="24"/>
-      <c r="R21" s="24"/>
-    </row>
-    <row r="22" s="19" customFormat="1" spans="1:14">
-      <c r="A22" s="25"/>
-      <c r="D22" s="19" t="s">
+      <c r="L21" s="37"/>
+      <c r="M21" s="37"/>
+      <c r="N21" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="O21" s="11"/>
+      <c r="P21" s="11"/>
+      <c r="Q21" s="11"/>
+      <c r="R21" s="11"/>
+    </row>
+    <row r="22" s="22" customFormat="1" spans="1:14">
+      <c r="A22" s="27"/>
+      <c r="D22" s="22" t="s">
         <v>136</v>
       </c>
-      <c r="E22" s="19" t="s">
+      <c r="E22" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="F22" s="19" t="s">
+      <c r="F22" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="H22" s="19" t="s">
+      <c r="H22" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="I22" s="19" t="s">
+      <c r="I22" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="J22" s="19" t="s">
+      <c r="J22" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="K22" s="36" t="s">
+      <c r="K22" s="38" t="s">
         <v>141</v>
       </c>
-      <c r="L22" s="37"/>
-      <c r="M22" s="37"/>
-      <c r="N22" s="19" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" s="19" customFormat="1" spans="1:17">
-      <c r="A23" s="25"/>
-      <c r="D23" s="19" t="s">
+      <c r="L22" s="39"/>
+      <c r="M22" s="39"/>
+      <c r="N22" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" s="22" customFormat="1" spans="1:17">
+      <c r="A23" s="27"/>
+      <c r="D23" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="E23" s="19" t="s">
+      <c r="E23" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="H23" s="19" t="s">
+      <c r="H23" s="22" t="s">
         <v>143</v>
       </c>
-      <c r="I23" s="19" t="s">
+      <c r="I23" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="J23" s="19" t="s">
+      <c r="J23" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="K23" s="36" t="s">
+      <c r="K23" s="38" t="s">
         <v>146</v>
       </c>
-      <c r="L23" s="37"/>
-      <c r="M23" s="37"/>
-      <c r="N23" s="19" t="b">
-        <v>1</v>
-      </c>
-      <c r="P23" s="19" t="s">
+      <c r="L23" s="39"/>
+      <c r="M23" s="39"/>
+      <c r="N23" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="P23" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="Q23" s="19" t="s">
+      <c r="Q23" s="22" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="24" s="19" customFormat="1" spans="1:17">
-      <c r="A24" s="25"/>
-      <c r="D24" s="19" t="s">
+    <row r="24" s="22" customFormat="1" spans="1:17">
+      <c r="A24" s="27"/>
+      <c r="D24" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="E24" s="19" t="s">
+      <c r="E24" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="H24" s="19" t="s">
+      <c r="H24" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="I24" s="19" t="s">
+      <c r="I24" s="22" t="s">
         <v>151</v>
       </c>
-      <c r="J24" s="19" t="s">
+      <c r="J24" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="K24" s="36" t="s">
+      <c r="K24" s="38" t="s">
         <v>153</v>
       </c>
-      <c r="L24" s="37"/>
-      <c r="M24" s="37"/>
-      <c r="P24" s="19" t="s">
+      <c r="L24" s="39"/>
+      <c r="M24" s="39"/>
+      <c r="P24" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="Q24" s="19" t="s">
+      <c r="Q24" s="22" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="25" s="20" customFormat="1" spans="1:15">
-      <c r="A25" s="26" t="s">
+    <row r="25" s="23" customFormat="1" spans="1:15">
+      <c r="A25" s="28" t="s">
         <v>154</v>
       </c>
-      <c r="D25" s="20" t="s">
+      <c r="D25" s="23" t="s">
         <v>155</v>
       </c>
-      <c r="E25" s="20" t="s">
+      <c r="E25" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="F25" s="29"/>
-      <c r="G25" s="29"/>
-      <c r="H25" s="20" t="s">
+      <c r="F25" s="31"/>
+      <c r="G25" s="31"/>
+      <c r="H25" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="I25" s="20" t="s">
+      <c r="I25" s="23" t="s">
         <v>158</v>
       </c>
-      <c r="J25" s="20" t="s">
+      <c r="J25" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="K25" s="38" t="s">
+      <c r="K25" s="40" t="s">
         <v>160</v>
       </c>
-      <c r="L25" s="39"/>
-      <c r="M25" s="39"/>
-      <c r="N25" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="O25" s="20" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" s="21" customFormat="1" spans="1:15">
-      <c r="A26" s="27" t="s">
+      <c r="L25" s="41"/>
+      <c r="M25" s="41"/>
+      <c r="N25" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="O25" s="23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" s="24" customFormat="1" spans="1:15">
+      <c r="A26" s="29" t="s">
         <v>154</v>
       </c>
-      <c r="D26" s="21" t="s">
+      <c r="D26" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="E26" s="21" t="s">
+      <c r="E26" s="24" t="s">
         <v>162</v>
       </c>
-      <c r="H26" s="21" t="s">
+      <c r="H26" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="I26" s="21" t="s">
+      <c r="I26" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="J26" s="21" t="s">
+      <c r="J26" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="K26" s="40" t="s">
+      <c r="K26" s="42" t="s">
         <v>166</v>
       </c>
-      <c r="L26" s="41"/>
-      <c r="M26" s="41"/>
-      <c r="N26" s="21" t="b">
-        <v>1</v>
-      </c>
-      <c r="O26" s="21" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" s="21" customFormat="1" spans="1:18">
-      <c r="A27" s="27" t="s">
+      <c r="L26" s="43"/>
+      <c r="M26" s="43"/>
+      <c r="N26" s="24" t="b">
+        <v>1</v>
+      </c>
+      <c r="O26" s="24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" s="24" customFormat="1" spans="1:18">
+      <c r="A27" s="29" t="s">
         <v>154</v>
       </c>
-      <c r="D27" s="21" t="s">
+      <c r="D27" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="E27" s="21" t="s">
+      <c r="E27" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="H27" s="21" t="s">
+      <c r="H27" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="I27" s="21" t="s">
+      <c r="I27" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="J27" s="21" t="s">
+      <c r="J27" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="K27" s="40" t="s">
+      <c r="K27" s="42" t="s">
         <v>170</v>
       </c>
-      <c r="L27" s="41"/>
-      <c r="M27" s="41"/>
-      <c r="O27" s="21" t="b">
-        <v>1</v>
-      </c>
-      <c r="R27" s="21" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" s="21" customFormat="1" spans="1:18">
-      <c r="A28" s="27" t="s">
+      <c r="L27" s="43"/>
+      <c r="M27" s="43"/>
+      <c r="O27" s="24" t="b">
+        <v>1</v>
+      </c>
+      <c r="R27" s="24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" s="24" customFormat="1" spans="1:18">
+      <c r="A28" s="29" t="s">
         <v>154</v>
       </c>
-      <c r="D28" s="21" t="s">
+      <c r="D28" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="E28" s="21" t="s">
+      <c r="E28" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="H28" s="21" t="s">
+      <c r="H28" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="I28" s="21" t="s">
+      <c r="I28" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="J28" s="21" t="s">
+      <c r="J28" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="K28" s="40" t="s">
+      <c r="K28" s="42" t="s">
         <v>173</v>
       </c>
-      <c r="L28" s="41"/>
-      <c r="M28" s="41"/>
-      <c r="O28" s="21" t="b">
-        <v>1</v>
-      </c>
-      <c r="R28" s="21" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" s="21" customFormat="1" spans="1:18">
-      <c r="A29" s="27" t="s">
+      <c r="L28" s="43"/>
+      <c r="M28" s="43"/>
+      <c r="O28" s="24" t="b">
+        <v>1</v>
+      </c>
+      <c r="R28" s="24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" s="24" customFormat="1" spans="1:18">
+      <c r="A29" s="29" t="s">
         <v>154</v>
       </c>
-      <c r="D29" s="21" t="s">
+      <c r="D29" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="E29" s="21" t="s">
+      <c r="E29" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="H29" s="21" t="s">
+      <c r="H29" s="24" t="s">
         <v>175</v>
       </c>
-      <c r="I29" s="21" t="s">
+      <c r="I29" s="24" t="s">
         <v>175</v>
       </c>
-      <c r="J29" s="21" t="s">
+      <c r="J29" s="24" t="s">
         <v>175</v>
       </c>
-      <c r="K29" s="40" t="s">
+      <c r="K29" s="42" t="s">
         <v>176</v>
       </c>
-      <c r="L29" s="41"/>
-      <c r="M29" s="41"/>
-      <c r="O29" s="21" t="b">
-        <v>1</v>
-      </c>
-      <c r="R29" s="21" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" s="22" customFormat="1" spans="1:15">
-      <c r="A30" s="28" t="s">
+      <c r="L29" s="43"/>
+      <c r="M29" s="43"/>
+      <c r="O29" s="24" t="b">
+        <v>1</v>
+      </c>
+      <c r="R29" s="24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" s="25" customFormat="1" spans="1:15">
+      <c r="A30" s="30" t="s">
         <v>154</v>
       </c>
-      <c r="D30" s="22" t="s">
+      <c r="D30" s="25" t="s">
         <v>177</v>
       </c>
-      <c r="E30" s="22" t="s">
+      <c r="E30" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="H30" s="22" t="s">
+      <c r="H30" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="I30" s="22" t="s">
+      <c r="I30" s="25" t="s">
         <v>179</v>
       </c>
-      <c r="J30" s="22" t="s">
+      <c r="J30" s="25" t="s">
         <v>180</v>
       </c>
-      <c r="K30" s="42" t="s">
+      <c r="K30" s="44" t="s">
         <v>181</v>
       </c>
-      <c r="L30" s="43"/>
-      <c r="M30" s="43"/>
-      <c r="N30" s="22" t="b">
-        <v>1</v>
-      </c>
-      <c r="O30" s="22" t="b">
+      <c r="L30" s="45"/>
+      <c r="M30" s="45"/>
+      <c r="N30" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="O30" s="25" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:13">
       <c r="A31" s="1"/>
-      <c r="K31" s="32"/>
-      <c r="L31" s="33"/>
-      <c r="M31" s="33"/>
+      <c r="K31" s="34"/>
+      <c r="L31" s="35"/>
+      <c r="M31" s="35"/>
     </row>
     <row r="32" spans="1:13">
       <c r="A32" s="1"/>
-      <c r="K32" s="33"/>
-      <c r="L32" s="33"/>
-      <c r="M32" s="33"/>
+      <c r="K32" s="35"/>
+      <c r="L32" s="35"/>
+      <c r="M32" s="35"/>
     </row>
     <row r="33" spans="1:13">
       <c r="A33" s="1"/>
-      <c r="K33" s="33"/>
-      <c r="L33" s="33"/>
-      <c r="M33" s="33"/>
+      <c r="K33" s="35"/>
+      <c r="L33" s="35"/>
+      <c r="M33" s="35"/>
     </row>
     <row r="34" spans="1:13">
       <c r="A34" s="1"/>
-      <c r="K34" s="33"/>
-      <c r="L34" s="33"/>
-      <c r="M34" s="33"/>
+      <c r="K34" s="35"/>
+      <c r="L34" s="35"/>
+      <c r="M34" s="35"/>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" s="1"/>
@@ -3230,7 +3237,8 @@
   <cols>
     <col min="1" max="1" width="12.5428571428571" customWidth="1"/>
     <col min="2" max="2" width="25.8190476190476" customWidth="1"/>
-    <col min="3" max="4" width="22.8190476190476" customWidth="1"/>
+    <col min="3" max="3" width="26.8" customWidth="1"/>
+    <col min="4" max="4" width="22.8190476190476" customWidth="1"/>
     <col min="5" max="5" width="37.1809523809524" customWidth="1"/>
     <col min="6" max="6" width="33.7047619047619" customWidth="1"/>
     <col min="7" max="7" width="13.1809523809524" customWidth="1"/>
@@ -3249,7 +3257,7 @@
       <c r="D1" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="14" t="s">
         <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -3272,10 +3280,10 @@
       <c r="D2" t="s">
         <v>184</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="14" t="s">
         <v>185</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G2" s="1"/>
@@ -3293,10 +3301,10 @@
       <c r="D3" t="s">
         <v>188</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="14" t="s">
         <v>189</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="15" t="s">
         <v>190</v>
       </c>
       <c r="G3" s="1"/>
@@ -3314,10 +3322,10 @@
       <c r="D4" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="16" t="s">
         <v>194</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="17" t="s">
         <v>195</v>
       </c>
       <c r="G4" s="3"/>
@@ -3335,10 +3343,10 @@
       <c r="D5" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="16" t="s">
         <v>199</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="17" t="s">
         <v>200</v>
       </c>
       <c r="G5" s="3"/>
@@ -3356,13 +3364,13 @@
       <c r="D6" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="16" t="s">
         <v>204</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="G6" s="19" t="s">
         <v>206</v>
       </c>
     </row>
@@ -3379,10 +3387,10 @@
       <c r="D7" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="20" t="s">
         <v>210</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="15" t="s">
         <v>211</v>
       </c>
     </row>
@@ -3399,10 +3407,10 @@
       <c r="D8" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="20" t="s">
         <v>215</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="15" t="s">
         <v>216</v>
       </c>
     </row>
@@ -3419,10 +3427,10 @@
       <c r="D9" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="E9" s="20" t="s">
         <v>220</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="15" t="s">
         <v>221</v>
       </c>
     </row>
@@ -3439,10 +3447,10 @@
       <c r="D10" s="7" t="s">
         <v>224</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="F10" s="15" t="s">
         <v>226</v>
       </c>
     </row>
@@ -3459,10 +3467,10 @@
       <c r="D11" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="20" t="s">
         <v>230</v>
       </c>
-      <c r="F11" s="12" t="s">
+      <c r="F11" s="15" t="s">
         <v>231</v>
       </c>
     </row>
@@ -3479,10 +3487,10 @@
       <c r="D12" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="20" t="s">
         <v>235</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="15" t="s">
         <v>236</v>
       </c>
     </row>
@@ -3499,10 +3507,10 @@
       <c r="D13" s="7" t="s">
         <v>239</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="20" t="s">
         <v>240</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="F13" s="15" t="s">
         <v>241</v>
       </c>
     </row>
@@ -3519,10 +3527,10 @@
       <c r="D14" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="20" t="s">
         <v>245</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="F14" s="15" t="s">
         <v>246</v>
       </c>
     </row>
@@ -3539,10 +3547,10 @@
       <c r="D15" t="s">
         <v>249</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="14" t="s">
         <v>250</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="F15" s="15" t="s">
         <v>251</v>
       </c>
     </row>
@@ -3559,10 +3567,10 @@
       <c r="D16" t="s">
         <v>254</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="14" t="s">
         <v>255</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="F16" s="15" t="s">
         <v>256</v>
       </c>
     </row>
@@ -3579,10 +3587,10 @@
       <c r="D17" t="s">
         <v>259</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="14" t="s">
         <v>260</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="F17" s="15" t="s">
         <v>261</v>
       </c>
     </row>
@@ -3599,10 +3607,10 @@
       <c r="D18" t="s">
         <v>264</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="14" t="s">
         <v>265</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="F18" s="15" t="s">
         <v>266</v>
       </c>
     </row>
@@ -3619,10 +3627,10 @@
       <c r="D19" t="s">
         <v>269</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="14" t="s">
         <v>270</v>
       </c>
-      <c r="F19" s="12" t="s">
+      <c r="F19" s="15" t="s">
         <v>271</v>
       </c>
     </row>
@@ -3639,10 +3647,10 @@
       <c r="D20" t="s">
         <v>274</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="14" t="s">
         <v>275</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="15" t="s">
         <v>276</v>
       </c>
     </row>
@@ -3659,10 +3667,10 @@
       <c r="D21" t="s">
         <v>279</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="14" t="s">
         <v>280</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="F21" s="15" t="s">
         <v>281</v>
       </c>
     </row>
@@ -3679,10 +3687,10 @@
       <c r="D22" t="s">
         <v>284</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="14" t="s">
         <v>285</v>
       </c>
-      <c r="F22" s="12" t="s">
+      <c r="F22" s="15" t="s">
         <v>286</v>
       </c>
     </row>
@@ -3699,10 +3707,10 @@
       <c r="D23" t="s">
         <v>289</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" s="14" t="s">
         <v>290</v>
       </c>
-      <c r="F23" s="12" t="s">
+      <c r="F23" s="15" t="s">
         <v>291</v>
       </c>
     </row>
@@ -3719,10 +3727,10 @@
       <c r="D24" t="s">
         <v>294</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="14" t="s">
         <v>295</v>
       </c>
-      <c r="F24" s="12" t="s">
+      <c r="F24" s="15" t="s">
         <v>296</v>
       </c>
     </row>
@@ -3739,10 +3747,10 @@
       <c r="D25" t="s">
         <v>299</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" s="14" t="s">
         <v>300</v>
       </c>
-      <c r="F25" s="12" t="s">
+      <c r="F25" s="15" t="s">
         <v>301</v>
       </c>
     </row>
@@ -3759,10 +3767,10 @@
       <c r="D26" t="s">
         <v>304</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="14" t="s">
         <v>305</v>
       </c>
-      <c r="F26" s="12" t="s">
+      <c r="F26" s="15" t="s">
         <v>306</v>
       </c>
     </row>
@@ -3779,10 +3787,10 @@
       <c r="D27" t="s">
         <v>309</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="14" t="s">
         <v>310</v>
       </c>
-      <c r="F27" s="18" t="s">
+      <c r="F27" s="21" t="s">
         <v>311</v>
       </c>
       <c r="G27" s="10"/>
@@ -3800,35 +3808,59 @@
       <c r="D28" t="s">
         <v>244</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" s="14" t="s">
         <v>245</v>
       </c>
-      <c r="F28" s="18" t="s">
+      <c r="F28" s="21" t="s">
         <v>313</v>
       </c>
       <c r="G28" s="10"/>
     </row>
     <row r="29" spans="1:7">
-      <c r="A29" s="8"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
+      <c r="A29" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="F29" s="12" t="s">
+        <v>314</v>
+      </c>
       <c r="G29" s="10"/>
     </row>
     <row r="30" spans="1:7">
-      <c r="A30" s="8"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
+      <c r="A30" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>314</v>
+      </c>
       <c r="G30" s="9"/>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="8"/>
-      <c r="B31" s="11"/>
+      <c r="B31" s="13"/>
       <c r="C31" s="10"/>
       <c r="D31" s="10"/>
       <c r="E31" s="10"/>
@@ -3837,7 +3869,7 @@
     </row>
     <row r="32" spans="1:7">
       <c r="A32" s="8"/>
-      <c r="B32" s="11"/>
+      <c r="B32" s="13"/>
       <c r="C32" s="10"/>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
@@ -3846,7 +3878,7 @@
     </row>
     <row r="33" spans="1:7">
       <c r="A33" s="8"/>
-      <c r="B33" s="11"/>
+      <c r="B33" s="13"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
       <c r="E33" s="10"/>
@@ -3855,7 +3887,7 @@
     </row>
     <row r="34" spans="1:7">
       <c r="A34" s="8"/>
-      <c r="B34" s="11"/>
+      <c r="B34" s="13"/>
       <c r="C34" s="10"/>
       <c r="D34" s="10"/>
       <c r="E34" s="10"/>
@@ -3864,7 +3896,7 @@
     </row>
     <row r="35" spans="1:7">
       <c r="A35" s="8"/>
-      <c r="B35" s="11"/>
+      <c r="B35" s="13"/>
       <c r="C35" s="10"/>
       <c r="D35" s="10"/>
       <c r="E35" s="10"/>
@@ -3873,7 +3905,7 @@
     </row>
     <row r="36" spans="1:7">
       <c r="A36" s="8"/>
-      <c r="B36" s="11"/>
+      <c r="B36" s="13"/>
       <c r="C36" s="10"/>
       <c r="D36" s="10"/>
       <c r="E36" s="10"/>
@@ -3882,7 +3914,7 @@
     </row>
     <row r="37" spans="1:7">
       <c r="A37" s="8"/>
-      <c r="B37" s="11"/>
+      <c r="B37" s="13"/>
       <c r="C37" s="10"/>
       <c r="D37" s="10"/>
       <c r="E37" s="10"/>
@@ -3891,7 +3923,7 @@
     </row>
     <row r="38" spans="1:7">
       <c r="A38" s="8"/>
-      <c r="B38" s="11"/>
+      <c r="B38" s="13"/>
       <c r="C38" s="10"/>
       <c r="D38" s="10"/>
       <c r="E38" s="10"/>
@@ -3900,7 +3932,7 @@
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="8"/>
-      <c r="B39" s="11"/>
+      <c r="B39" s="13"/>
       <c r="C39" s="10"/>
       <c r="D39" s="10"/>
       <c r="E39" s="10"/>
@@ -3909,7 +3941,7 @@
     </row>
     <row r="40" spans="1:7">
       <c r="A40" s="8"/>
-      <c r="B40" s="11"/>
+      <c r="B40" s="13"/>
       <c r="C40" s="10"/>
       <c r="D40" s="10"/>
       <c r="E40" s="10"/>
@@ -3974,27 +4006,27 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C1" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E1" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C2" t="s">
         <v>254</v>
@@ -4003,7 +4035,7 @@
         <v>255</v>
       </c>
       <c r="E2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>

</xml_diff>